<commit_message>
feat(recursos): animacao Controladoria, FP&A e Tesouraria e ajustes de conteudo
- nova animacao controladoria_fpa_tesouraria como primeiro card do Modulo 1
- cenario "Mesa de juros" do breakeven cita a diferenca como premio + liquidez
- planilha de revisao de matematica financeira atualizada

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/simulacoes/revisao-modelos-matematica-financeira.xlsx
+++ b/public/simulacoes/revisao-modelos-matematica-financeira.xlsx
@@ -5,20 +5,25 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Disciplinas\FGV - Disciplinas\Operações de Tesouraria em IFs\Avaliações\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\jose_americo\laboratorio-tesouraria_IFs\simmulations\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C2A386-85B0-4C82-84B6-A6CF47FDDD4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BD7A476-5FE5-4373-BAC0-D19D77702749}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{BF4D0276-6DDD-4177-BBA4-BABB450DE40C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="6" activeTab="9" xr2:uid="{BF4D0276-6DDD-4177-BBA4-BABB450DE40C}"/>
   </bookViews>
   <sheets>
     <sheet name="Início" sheetId="1" r:id="rId1"/>
-    <sheet name="1. VP e VF" sheetId="2" r:id="rId2"/>
-    <sheet name="2. Equivalência" sheetId="3" r:id="rId3"/>
-    <sheet name="3. LTN (zero-cupom)" sheetId="4" r:id="rId4"/>
-    <sheet name="4. Fluxo com cupons" sheetId="5" r:id="rId5"/>
-    <sheet name="5. TIR e YTM" sheetId="6" r:id="rId6"/>
+    <sheet name="1. VP e VF (aula)" sheetId="7" r:id="rId2"/>
+    <sheet name="1. VP e VF" sheetId="2" r:id="rId3"/>
+    <sheet name="2. Equivalência (aula)" sheetId="8" r:id="rId4"/>
+    <sheet name="2. Equivalência" sheetId="3" r:id="rId5"/>
+    <sheet name="3. LTN (zero-cupom) (aula)" sheetId="9" r:id="rId6"/>
+    <sheet name="3. LTN (zero-cupom)" sheetId="4" r:id="rId7"/>
+    <sheet name="4. Fluxo com cupons (aula)" sheetId="10" r:id="rId8"/>
+    <sheet name="4. Fluxo com cupons" sheetId="5" r:id="rId9"/>
+    <sheet name="5. TIR e YTM (aula)" sheetId="11" r:id="rId10"/>
+    <sheet name="5. TIR e YTM" sheetId="6" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="105">
   <si>
     <t>Simulador 1 — Valor do dinheiro no tempo (VP ↔ VF)</t>
   </si>
@@ -1057,7 +1062,987 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9936388-F3EF-47E1-AA2B-353A3E1A4060}">
+  <dimension ref="A1:H33"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="42.5546875" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="3.6640625" customWidth="1"/>
+    <col min="4" max="4" width="81.44140625" customWidth="1"/>
+    <col min="5" max="6" width="3.6640625" customWidth="1"/>
+    <col min="7" max="7" width="11.109375" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" s="27">
+        <v>893.24</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" s="13">
+        <v>0</v>
+      </c>
+      <c r="H3" s="29">
+        <f>-B3</f>
+        <v>-893.24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" s="27">
+        <v>120</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="G4" s="13">
+        <f>G3+1</f>
+        <v>1</v>
+      </c>
+      <c r="H4" s="29">
+        <f>IF(ROW()-3&gt;$B$5,"",$B$4+IF(ROW()-3=$B$5,$B$6,0))</f>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="5">
+        <v>5</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="G5" s="13">
+        <f t="shared" ref="G5:G33" si="0">G4+1</f>
+        <v>2</v>
+      </c>
+      <c r="H5" s="29">
+        <f t="shared" ref="H5:H33" si="1">IF(ROW()-3&gt;$B$5,"",$B$4+IF(ROW()-3=$B$5,$B$6,0))</f>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="27">
+        <v>1000</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="G6" s="13">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H6" s="29">
+        <f t="shared" si="1"/>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="3"/>
+      <c r="D7" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="G7" s="13">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H7" s="29">
+        <f t="shared" si="1"/>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="16"/>
+      <c r="D8" s="8"/>
+      <c r="G8" s="13">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H8" s="29">
+        <f t="shared" si="1"/>
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="17">
+        <f>B8</f>
+        <v>0</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="13">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="H9" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>85</v>
+      </c>
+      <c r="G10" s="13">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="H10" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D11" t="s">
+        <v>86</v>
+      </c>
+      <c r="G11" s="13">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="H11" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>87</v>
+      </c>
+      <c r="G12" s="13">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="H12" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G13" s="13">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="H13" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D14" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G14" s="13">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="H14" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G15" s="13">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="H15" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G16" s="13">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="H16" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G17" s="13">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="H17" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G18" s="13">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="H18" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G19" s="13">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="H19" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G20" s="13">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="H20" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G21" s="13">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="H21" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G22" s="13">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="H22" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G23" s="13">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="H23" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G24" s="13">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="H24" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G25" s="13">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="H25" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G26" s="13">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="H26" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G27" s="13">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="H27" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G28" s="13">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="H28" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G29" s="13">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="H29" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G30" s="13">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+      <c r="H30" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G31" s="13">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="H31" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G32" s="13">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+      <c r="H32" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G33" s="13">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="H33" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Nº de anos inválido" error="O número de anos deve ser um inteiro entre 1 e 30." sqref="B5" xr:uid="{C88680BA-9356-4A9D-8456-BE60A33229EF}">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Digite um valor monetário maior que zero." sqref="B6 B3:B4" xr:uid="{03E35133-5A23-4E35-8566-711C1D37EB55}">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{278690ED-91A0-40C4-89D6-0029F43B2843}">
+  <dimension ref="A1:H33"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="42.5546875" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="3.6640625" customWidth="1"/>
+    <col min="4" max="4" width="81.44140625" customWidth="1"/>
+    <col min="5" max="6" width="3.6640625" customWidth="1"/>
+    <col min="7" max="7" width="11.109375" customWidth="1"/>
+    <col min="8" max="8" width="25.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="H2" s="12" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" s="27">
+        <v>893.24</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" s="13">
+        <v>0</v>
+      </c>
+      <c r="H3" s="29">
+        <f>-B3</f>
+        <v>-893.24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4" s="27">
+        <v>120</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="G4" s="13">
+        <f>G3+1</f>
+        <v>1</v>
+      </c>
+      <c r="H4" s="29">
+        <f>IF(ROW()-3&gt;$B$5,"",$B$4+IF(ROW()-3=$B$5,$B$6,0))</f>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5" s="5">
+        <v>5</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="G5" s="13">
+        <f t="shared" ref="G5:G33" si="0">G4+1</f>
+        <v>2</v>
+      </c>
+      <c r="H5" s="29">
+        <f t="shared" ref="H5:H33" si="1">IF(ROW()-3&gt;$B$5,"",$B$4+IF(ROW()-3=$B$5,$B$6,0))</f>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="27">
+        <v>1000</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="G6" s="13">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="H6" s="29">
+        <f t="shared" si="1"/>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="3"/>
+      <c r="D7" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="G7" s="13">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H7" s="29">
+        <f t="shared" si="1"/>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="18" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="16">
+        <f>IRR(H3:H33)</f>
+        <v>0.15199903923974278</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="G8" s="13">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="H8" s="29">
+        <f t="shared" si="1"/>
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="17">
+        <f>B8</f>
+        <v>0.15199903923974278</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" s="13">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="H9" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>85</v>
+      </c>
+      <c r="G10" s="13">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="H10" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D11" t="s">
+        <v>86</v>
+      </c>
+      <c r="G11" s="13">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="H11" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>87</v>
+      </c>
+      <c r="G12" s="13">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="H12" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G13" s="13">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="H13" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="D14" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G14" s="13">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="H14" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G15" s="13">
+        <f t="shared" si="0"/>
+        <v>12</v>
+      </c>
+      <c r="H15" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G16" s="13">
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="H16" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G17" s="13">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="H17" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G18" s="13">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="H18" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G19" s="13">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="H19" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G20" s="13">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="H20" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G21" s="13">
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="H21" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G22" s="13">
+        <f t="shared" si="0"/>
+        <v>19</v>
+      </c>
+      <c r="H22" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G23" s="13">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="H23" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G24" s="13">
+        <f t="shared" si="0"/>
+        <v>21</v>
+      </c>
+      <c r="H24" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G25" s="13">
+        <f t="shared" si="0"/>
+        <v>22</v>
+      </c>
+      <c r="H25" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G26" s="13">
+        <f t="shared" si="0"/>
+        <v>23</v>
+      </c>
+      <c r="H26" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G27" s="13">
+        <f t="shared" si="0"/>
+        <v>24</v>
+      </c>
+      <c r="H27" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G28" s="13">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="H28" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G29" s="13">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="H29" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G30" s="13">
+        <f t="shared" si="0"/>
+        <v>27</v>
+      </c>
+      <c r="H30" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G31" s="13">
+        <f t="shared" si="0"/>
+        <v>28</v>
+      </c>
+      <c r="H31" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G32" s="13">
+        <f t="shared" si="0"/>
+        <v>29</v>
+      </c>
+      <c r="H32" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G33" s="13">
+        <f t="shared" si="0"/>
+        <v>30</v>
+      </c>
+      <c r="H33" s="29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Digite um valor monetário maior que zero." sqref="B6 B3:B4" xr:uid="{C9FF1A67-CE16-4795-88BC-3541F0B94528}">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Nº de anos inválido" error="O número de anos deve ser um inteiro entre 1 e 30." sqref="B5" xr:uid="{7A8A86AD-6376-4300-8CF8-421C76080878}">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45F8C813-861B-4D45-8265-CFE47443D2F8}">
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="42.5546875" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="3.6640625" customWidth="1"/>
+    <col min="4" max="4" width="79.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="25">
+        <v>100000</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="23">
+        <v>0.12</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="24">
+        <v>21</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="22"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="30"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="3"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="26"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="26"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Prazo inválido" error="O prazo em dias úteis deve ser um número inteiro maior ou igual a 1." sqref="B5" xr:uid="{E25E473C-DFBA-4DFF-883F-A5527D9274DF}">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Taxa inválida" error="Digite uma taxa entre 0% e 100%." sqref="B4" xr:uid="{FA27DB35-D2B5-42F9-BDD8-0FEAF94568E5}">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Digite um valor monetário maior que zero." sqref="B3" xr:uid="{3C046DFF-973A-4E46-85E6-90D81094E5F3}">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F98024E5-FB32-4149-8C8E-3ED618521C8C}">
   <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1200,7 +2185,172 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A539789-34F1-43C8-8410-151F303F3E8E}">
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="48.109375" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="3.6640625" customWidth="1"/>
+    <col min="4" max="4" width="79.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="4">
+        <v>0.12</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" s="5">
+        <v>21</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="3"/>
+      <c r="D5" s="8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="30"/>
+      <c r="D6" s="8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="30"/>
+      <c r="D7" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="30"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="30"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="3"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="4">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" s="9">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="3"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B15" s="30"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="6"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="6"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Prazo inválido" error="O prazo em dias úteis deve ser um número inteiro maior ou igual a 1." sqref="B4" xr:uid="{35F8CF27-9B26-4B32-95BE-FF0899D91C53}">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Percentual inválido" error="Digite um percentual entre 0% e 500%." sqref="B13" xr:uid="{7286C941-1FC4-45B1-8ABF-7744783073B9}">
+      <formula1>0</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Taxa inválida" error="Digite uma taxa entre 0% e 100%." sqref="B3 B12" xr:uid="{6E87A73A-7691-44F6-850F-4CBC0DBF476E}">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D93EAB39-514D-471C-932F-7EB9C6047A5D}">
   <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1386,7 +2536,160 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874683C5-8EBF-4317-8C35-7A4569FC3741}">
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="48.109375" customWidth="1"/>
+    <col min="2" max="2" width="20.33203125" customWidth="1"/>
+    <col min="3" max="3" width="3.6640625" customWidth="1"/>
+    <col min="4" max="4" width="79.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="27">
+        <v>1000</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4">
+        <v>0.13500000000000001</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5">
+        <v>252</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="3"/>
+      <c r="D6" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="26"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" s="26"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="3"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B11" s="27">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B12" s="5">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" s="27">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="3"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" s="6"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Prazo inválido" error="O prazo em dias úteis deve ser um número inteiro maior ou igual a 1." sqref="B5 B12" xr:uid="{BCCC6BCB-E04B-4EAE-AC31-A720D52570B4}">
+      <formula1>1</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Taxa inválida" error="Digite uma taxa entre 0% e 100%." sqref="B4" xr:uid="{DDE1380F-4D2D-4A19-B09D-690E15ADC9AE}">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Digite um valor monetário maior que zero." sqref="B3 B13 B11" xr:uid="{733BBB16-1A60-4660-BC30-FC7AE4408C85}">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CED07BA4-A75B-4DC3-A02B-CA500D0CB420}">
   <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1548,7 +2851,669 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BF785F8-B870-48A1-BF9A-C29A75F45690}">
+  <dimension ref="A1:F40"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22.88671875" customWidth="1"/>
+    <col min="2" max="4" width="22.21875" customWidth="1"/>
+    <col min="5" max="5" width="40.77734375" customWidth="1"/>
+    <col min="6" max="6" width="81.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="27">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" s="4">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="5">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B6" s="4">
+        <v>0.152</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="3"/>
+      <c r="E7" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="18" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" s="26">
+        <f>B3*B4</f>
+        <v>120</v>
+      </c>
+      <c r="F8" s="31">
+        <f>SUM(D11:D40)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="13">
+        <v>1</v>
+      </c>
+      <c r="B11" s="28">
+        <f>IF(A11&gt;$B$5,"",$B$8+IF(A11=$B$5,$B$3,0))</f>
+        <v>120</v>
+      </c>
+      <c r="C11" s="14">
+        <f>IF(A11&gt;$B$5,"",(1+$B$6)^A11)</f>
+        <v>1.1519999999999999</v>
+      </c>
+      <c r="D11" s="29"/>
+      <c r="F11" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="13">
+        <f>A11+1</f>
+        <v>2</v>
+      </c>
+      <c r="B12" s="28">
+        <f t="shared" ref="B12:B40" si="0">IF(A12&gt;$B$5,"",$B$8+IF(A12=$B$5,$B$3,0))</f>
+        <v>120</v>
+      </c>
+      <c r="C12" s="14">
+        <f t="shared" ref="C12:C40" si="1">IF(A12&gt;$B$5,"",(1+$B$6)^A12)</f>
+        <v>1.3271039999999998</v>
+      </c>
+      <c r="D12" s="29"/>
+      <c r="F12" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="13">
+        <f t="shared" ref="A13:A40" si="2">A12+1</f>
+        <v>3</v>
+      </c>
+      <c r="B13" s="28">
+        <f t="shared" si="0"/>
+        <v>120</v>
+      </c>
+      <c r="C13" s="14">
+        <f t="shared" si="1"/>
+        <v>1.5288238079999996</v>
+      </c>
+      <c r="D13" s="29"/>
+      <c r="F13" s="8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="13">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="B14" s="28">
+        <f t="shared" si="0"/>
+        <v>120</v>
+      </c>
+      <c r="C14" s="14">
+        <f t="shared" si="1"/>
+        <v>1.7612050268159996</v>
+      </c>
+      <c r="D14" s="29"/>
+      <c r="F14" s="8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="13">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="B15" s="28">
+        <f t="shared" si="0"/>
+        <v>1120</v>
+      </c>
+      <c r="C15" s="14">
+        <f t="shared" si="1"/>
+        <v>2.0289081908920314</v>
+      </c>
+      <c r="D15" s="29"/>
+      <c r="F15" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="13">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="B16" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C16" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D16" s="29" t="str">
+        <f t="shared" ref="D12:D40" si="3">IF(A16&gt;$B$5,"",B16/C16)</f>
+        <v/>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="13">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="B17" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C17" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D17" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="13">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="B18" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C18" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D18" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F18" s="8"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="13">
+        <f t="shared" si="2"/>
+        <v>9</v>
+      </c>
+      <c r="B19" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C19" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D19" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="13">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
+      <c r="B20" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C20" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D20" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F20" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="13">
+        <f t="shared" si="2"/>
+        <v>11</v>
+      </c>
+      <c r="B21" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C21" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D21" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F21" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="13">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="B22" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C22" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D22" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="13">
+        <f t="shared" si="2"/>
+        <v>13</v>
+      </c>
+      <c r="B23" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C23" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D23" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="13">
+        <f t="shared" si="2"/>
+        <v>14</v>
+      </c>
+      <c r="B24" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C24" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D24" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="13">
+        <f t="shared" si="2"/>
+        <v>15</v>
+      </c>
+      <c r="B25" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C25" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D25" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="13">
+        <f t="shared" si="2"/>
+        <v>16</v>
+      </c>
+      <c r="B26" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C26" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D26" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="13">
+        <f t="shared" si="2"/>
+        <v>17</v>
+      </c>
+      <c r="B27" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C27" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D27" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="13">
+        <f t="shared" si="2"/>
+        <v>18</v>
+      </c>
+      <c r="B28" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C28" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D28" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="13">
+        <f t="shared" si="2"/>
+        <v>19</v>
+      </c>
+      <c r="B29" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C29" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D29" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="13">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
+      <c r="B30" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C30" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D30" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="13">
+        <f t="shared" si="2"/>
+        <v>21</v>
+      </c>
+      <c r="B31" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C31" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D31" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="13">
+        <f t="shared" si="2"/>
+        <v>22</v>
+      </c>
+      <c r="B32" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C32" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D32" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="13">
+        <f t="shared" si="2"/>
+        <v>23</v>
+      </c>
+      <c r="B33" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C33" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D33" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="13">
+        <f t="shared" si="2"/>
+        <v>24</v>
+      </c>
+      <c r="B34" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C34" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D34" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="13">
+        <f t="shared" si="2"/>
+        <v>25</v>
+      </c>
+      <c r="B35" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C35" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D35" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="13">
+        <f t="shared" si="2"/>
+        <v>26</v>
+      </c>
+      <c r="B36" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C36" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D36" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="13">
+        <f t="shared" si="2"/>
+        <v>27</v>
+      </c>
+      <c r="B37" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C37" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D37" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="13">
+        <f t="shared" si="2"/>
+        <v>28</v>
+      </c>
+      <c r="B38" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C38" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D38" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="13">
+        <f t="shared" si="2"/>
+        <v>29</v>
+      </c>
+      <c r="B39" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C39" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D39" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" s="13">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
+      <c r="B40" s="28" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="C40" s="14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="D40" s="29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Nº de anos inválido" error="O número de anos deve ser um inteiro entre 1 e 30." sqref="B5" xr:uid="{64A52C0C-E697-4D41-9F99-4E04B4CD1BAE}">
+      <formula1>1</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Taxa inválida" error="Digite uma taxa entre 0% e 100%." sqref="B4 B6" xr:uid="{03471D33-1132-49E5-81AF-04B2D7B49800}">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
+    </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Digite um valor monetário maior que zero." sqref="B3" xr:uid="{05E7EA9E-2B63-4F0C-BD1F-7BF9FA14620E}">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65333286-B62B-45DE-8150-BF5A3E0278CF}">
   <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2223,430 +4188,4 @@
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{278690ED-91A0-40C4-89D6-0029F43B2843}">
-  <dimension ref="A1:H33"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="42.5546875" customWidth="1"/>
-    <col min="2" max="2" width="20.33203125" customWidth="1"/>
-    <col min="3" max="3" width="3.6640625" customWidth="1"/>
-    <col min="4" max="4" width="81.44140625" customWidth="1"/>
-    <col min="5" max="6" width="3.6640625" customWidth="1"/>
-    <col min="7" max="7" width="11.109375" customWidth="1"/>
-    <col min="8" max="8" width="25.88671875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="H2" s="12" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B3" s="27">
-        <v>893.24</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="G3" s="13">
-        <v>0</v>
-      </c>
-      <c r="H3" s="29">
-        <f>-B3</f>
-        <v>-893.24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B4" s="27">
-        <v>120</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="G4" s="13">
-        <f>G3+1</f>
-        <v>1</v>
-      </c>
-      <c r="H4" s="29">
-        <f>IF(ROW()-3&gt;$B$5,"",$B$4+IF(ROW()-3=$B$5,$B$6,0))</f>
-        <v>120</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B5" s="5">
-        <v>5</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="G5" s="13">
-        <f t="shared" ref="G5:G33" si="0">G4+1</f>
-        <v>2</v>
-      </c>
-      <c r="H5" s="29">
-        <f t="shared" ref="H5:H33" si="1">IF(ROW()-3&gt;$B$5,"",$B$4+IF(ROW()-3=$B$5,$B$6,0))</f>
-        <v>120</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B6" s="27">
-        <v>1000</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="G6" s="13">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="H6" s="29">
-        <f t="shared" si="1"/>
-        <v>120</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="3"/>
-      <c r="D7" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="G7" s="13">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="H7" s="29">
-        <f t="shared" si="1"/>
-        <v>120</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="B8" s="16">
-        <f>IRR(H3:H33)</f>
-        <v>0.15199903923974278</v>
-      </c>
-      <c r="D8" s="8"/>
-      <c r="G8" s="13">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="H8" s="29">
-        <f t="shared" si="1"/>
-        <v>1120</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="B9" s="17">
-        <f>B8</f>
-        <v>0.15199903923974278</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="G9" s="13">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="H9" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D10" t="s">
-        <v>85</v>
-      </c>
-      <c r="G10" s="13">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="H10" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D11" t="s">
-        <v>86</v>
-      </c>
-      <c r="G11" s="13">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="H11" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D12" t="s">
-        <v>87</v>
-      </c>
-      <c r="G12" s="13">
-        <f t="shared" si="0"/>
-        <v>9</v>
-      </c>
-      <c r="H12" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G13" s="13">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="H13" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D14" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="G14" s="13">
-        <f t="shared" si="0"/>
-        <v>11</v>
-      </c>
-      <c r="H14" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G15" s="13">
-        <f t="shared" si="0"/>
-        <v>12</v>
-      </c>
-      <c r="H15" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="G16" s="13">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="H16" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="17" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G17" s="13">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="H17" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="18" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G18" s="13">
-        <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="H18" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="19" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G19" s="13">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="H19" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G20" s="13">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-      <c r="H20" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G21" s="13">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-      <c r="H21" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G22" s="13">
-        <f t="shared" si="0"/>
-        <v>19</v>
-      </c>
-      <c r="H22" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G23" s="13">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="H23" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G24" s="13">
-        <f t="shared" si="0"/>
-        <v>21</v>
-      </c>
-      <c r="H24" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G25" s="13">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
-      <c r="H25" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="26" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G26" s="13">
-        <f t="shared" si="0"/>
-        <v>23</v>
-      </c>
-      <c r="H26" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G27" s="13">
-        <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
-      <c r="H27" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G28" s="13">
-        <f t="shared" si="0"/>
-        <v>25</v>
-      </c>
-      <c r="H28" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G29" s="13">
-        <f t="shared" si="0"/>
-        <v>26</v>
-      </c>
-      <c r="H29" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G30" s="13">
-        <f t="shared" si="0"/>
-        <v>27</v>
-      </c>
-      <c r="H30" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G31" s="13">
-        <f t="shared" si="0"/>
-        <v>28</v>
-      </c>
-      <c r="H31" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G32" s="13">
-        <f t="shared" si="0"/>
-        <v>29</v>
-      </c>
-      <c r="H32" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="33" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G33" s="13">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-      <c r="H33" s="29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor inválido" error="Digite um valor monetário maior que zero." sqref="B6 B3:B4" xr:uid="{C9FF1A67-CE16-4795-88BC-3541F0B94528}">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Nº de anos inválido" error="O número de anos deve ser um inteiro entre 1 e 30." sqref="B5" xr:uid="{7A8A86AD-6376-4300-8CF8-421C76080878}">
-      <formula1>1</formula1>
-      <formula2>30</formula2>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
 </file>
</xml_diff>